<commit_message>
feat(recipes): polish reviewed catalog and thumbnails
</commit_message>
<xml_diff>
--- a/data/content-review-batches/12_rows_111-120.xlsx
+++ b/data/content-review-batches/12_rows_111-120.xlsx
@@ -390,8 +390,7 @@
 נערבב את הירקות ביחד עם כל הרכיבים 
 נחלק ל25 קציצות 
 נאפה בתנור שחומם מראש על 180 מעלות טורבו ל20-25 דקות (תלוי בתנור) 
-ובתאבון ✨✨
-#דלקלוריות</x:t>
+ובתאבון ✨✨</x:t>
         </x:is>
       </x:c>
       <x:c r="J2" t="inlineStr">
@@ -469,15 +468,13 @@
         <x:is>
           <x:t xml:space="preserve">אופן הכנה:
 נערבב את כל המצרכים בקערה אחת נמזוג לתבנית 20*20
-נאפה בתנור שחומם מראש על חום של 150 מעלות סטטי לשעה ורבע 
-•בתחתית התנור נשים תבנית עם מים רותחים
-נשאיר את העוגה בתנור סגור לפחות שעתיים (לא לפתוח במהלך האפייה) 
+נאפה בתנור שחומם מראש על חום של 150 מעלות סטטי לשעה ורבע
+בתחתית התנור נשים תבנית עם מים רותחים
+נשאיר את העוגה בתנור סגור לפחות שעתיים (לא לפתוח במהלך האפייה)
 ואז לעוד לילה במקרר ובתיאבון❤️❤️
-חילקתי את העוגה ל16 חתיכות 
-עם תחליף סוכר:
-כל חתיכה 94 קלוריות ו6 גרם חלבון 
-בלי תחליף סוכר: 
-כל חתיכה 131 קלוריות ו6 גרם חלבון</x:t>
+חילקתי את העוגה ל16 חתיכות
+עם תחליף סוכר: כל חתיכה 94 קלוריות ו6 גרם חלבון
+בלי תחליף סוכר: כל חתיכה 131 קלוריות ו6 גרם חלבון</x:t>
         </x:is>
       </x:c>
       <x:c r="J3" t="inlineStr">
@@ -564,10 +561,13 @@
 פטרוזיליה</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>אופן ההכנה:
+        <x:is>
+          <x:t xml:space="preserve">אופן ההכנה:
 קוצצים את הבצל, הגזר והסלרי. מטגנים את הבצל בשמן זית, מוסיפים את הסלרי והגזר, ולאחר מכן את הבשר. כשהבשר משנה צבע מוסיפים רסק עגבניות, פפריקה, מלח, פלפל, עגבניות מרוסקות ויין אדום, ומבשלים 10 דקות.
 לרוטב: מטגנים את השום בשמן זית, מוסיפים פפריקה, מלח, פלפל, עגבניות מרוסקות ומים, ומבשלים 10 דקות.
-ממלאים 11–12 קנלוני בבשר. יוצקים שליש מהרוטב לתבנית, מסדרים את הקנלוני ומכסים ביתרת הרוטב. מכסים בנייר כסף ואופים ב־180 מעלות טורבו 40 דקות. מסירים את הכיסוי ואופים עוד 5 דקות. מפזרים פטרוזיליה.</x:v>
+ממלאים 11–12 קנלוני בבשר. יוצקים שליש מהרוטב לתבנית, מסדרים את הקנלוני ומכסים ביתרת הרוטב.
+מכסים בנייר כסף ואופים ב־180 מעלות טורבו 40 דקות. מסירים את הכיסוי ואופים עוד 5 דקות. מפזרים פטרוזיליה.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>COMPLETE</x:v>
@@ -584,12 +584,12 @@
       </x:c>
       <x:c r="M4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">בינוני</x:t>
         </x:is>
       </x:c>
       <x:c r="N4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">90</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -735,19 +735,17 @@
       </x:c>
       <x:c r="I6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">הכנת הבצק פריך: 
-במיקסר עם וו גיטרה נשים את האבקת סוכר והחמאה ונפעיל עד לאיחוד 
-נוסיף את הקמח והקורנפלור ונעבד עד מרקם חולי,נוסיף את הביצה עד שמתגבש לבצק 
-•במידה ותשתמשו בביצה קטנה מדי הבצק לא יתאחד אז במידת הצורך אפשר להוסיף כפית חלב 
-נרדד למלבן גדול נמרח נוטלה ונסדר את המרשמלו 
-נגלגל את הבצק כמו בסרטון לגליל ארוך ונקפיא אותו למשך 40-60 דקות 
-נוציא את הגליל מהמקפיא ונניח על תבנית עם נייר אפייה ונאפה 20-25 דקות/ עד שהבצק מזהיב 
-בתנור שחומם מראש על 170 מעלות טורבו 
-נוציא מהתנור ונצנן בחוץ עד שמתקרר לגמרי 
-נבזוק אבקת סוכר ונפרוס פרוסות באופן שווה 
+          <x:t xml:space="preserve">הכנת הבצק פריך: במיקסר עם וו גיטרה נשים את האבקת סוכר והחמאה ונפעיל עד לאיחוד
+נוסיף את הקמח והקורנפלור ונעבד עד מרקם חולי,נוסיף את הביצה עד שמתגבש לבצק
+במידה ותשתמשו בביצה קטנה מדי הבצק לא יתאחד אז במידת הצורך אפשר להוסיף כפית חלב
+נרדד למלבן גדול נמרח נוטלה ונסדר את המרשמלו
+נגלגל את הבצק כמו בסרטון לגליל ארוך ונקפיא אותו למשך 40-60 דקות
+נוציא את הגליל מהמקפיא ונניח על תבנית עם נייר אפייה ונאפה 20-25 דקות/ עד שהבצק מזהיב
+בתנור שחומם מראש על 170 מעלות טורבו
+נוציא מהתנור ונצנן בחוץ עד שמתקרר לגמרי
+נבזוק אבקת סוכר ונפרוס פרוסות באופן שווה
 ובתיאבון ❤️❤️❤️
-שימו לב:
-בגלל שבזמן אפייה המרשמלו מתנפח אז באמצע הגליל יווצר לכם סדק וזה בסדר 🫶🏼</x:t>
+שימו לב: בגלל שבזמן אפייה המרשמלו מתנפח אז באמצע הגליל יווצר לכם סדק וזה בסדר 🫶🏼</x:t>
         </x:is>
       </x:c>
       <x:c r="J6" t="inlineStr">
@@ -918,32 +916,29 @@
       </x:c>
       <x:c r="I8" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">אופן הכנת הבצק: 
-בקערת מיקסר נשים קמח שמרים וסוכר ונערבב דקה (אפשר גם לערבב עם כף) 
-אחר כך נוסיף את הביצה, השמנת והחלב 
-ונלוש 5 דקות 
-אחרי שנראה שהבצק מתאחד נוסיף בהדרגה את החמאה 
-(נחתוך את החמאה לקוביות קטנות וכל כמה שניות נוסיף קוביית חמאה) 
-אחרי שכל החמאה נטמעה בבצק (בין 4-5 דקות) 
-נוסיף את המלח ונלוש עוד 3 דקות. 
-שימו לב- 
-זמן הלישה משתנה בין מיקסר למיקסר כי לפעמים יש מיקסרים פחות חזקים 
+          <x:t xml:space="preserve">אופן הכנת הבצק: בקערת מיקסר נשים קמח שמרים וסוכר ונערבב דקה (אפשר גם לערבב עם כף)
+אחר כך נוסיף את הביצה, השמנת והחלב
+ונלוש 5 דקות
+אחרי שנראה שהבצק מתאחד נוסיף בהדרגה את החמאה
+(נחתוך את החמאה לקוביות קטנות וכל כמה שניות נוסיף קוביית חמאה)
+אחרי שכל החמאה נטמעה בבצק (בין 4-5 דקות)
+נוסיף את המלח ונלוש עוד 3 דקות.
+שימו לב- זמן הלישה משתנה בין מיקסר למיקסר כי לפעמים יש מיקסרים פחות חזקים
 3 דקות אחרי שהוספתם את המלח כדי לבדוק אם הבצק סיים את הלישה תבדקו האם יש בבצק רשת גלוטן (בהייליט טיפים אצלי בעמוד אני מראה איך בודקים)
-אם אתם לא בטוחים עדיף ללוש את הבצק עוד כמה דקות. 
-אחרי שהבצק סיים את הלישה שלו נניח אותו בקערה משומנת. 
-עכשיו יש 2 אופציות 
-אופציה 1- לשים את הבצק בהתפחה של לילה במקרר ואז למחרת שעה לפני שרוצים לעבוד איתו להוציא אותו לטמפרטורת החדר ורק אז לעבוד איתו 
-זאת האופציה העדיפה כי ככה הבצק תופח יותר טוב ויותר נוח לעבוד איתו 
-אופציה 2- 
-אם אין לכם זמן להתפחת לילה תתפיחו בחוץ שעה- שעה וחצי עד שהבצק מכפיל את עצמו 
-אחרי שהבצק סיים לתפוח נחלק אותו ל2 חלקים שווים 
-נקח את החלק הראשון למלבן עבה ולא גדול ובעזרת גלגלת פיצה נחתוך לריבועים 
-כל ריבוע נגלגל לכדור 
+אם אתם לא בטוחים עדיף ללוש את הבצק עוד כמה דקות.
+אחרי שהבצק סיים את הלישה שלו נניח אותו בקערה משומנת.
+עכשיו יש 2 אופציות
+אופציה 1- לשים את הבצק בהתפחה של לילה במקרר ואז למחרת שעה לפני שרוצים לעבוד איתו להוציא אותו לטמפרטורת החדר ורק אז לעבוד איתו
+זאת האופציה העדיפה כי ככה הבצק תופח יותר טוב ויותר נוח לעבוד איתו
+אופציה 2- אם אין לכם זמן להתפחת לילה תתפיחו בחוץ שעה- שעה וחצי עד שהבצק מכפיל את עצמו
+אחרי שהבצק סיים לתפוח נחלק אותו ל2 חלקים שווים
+נקח את החלק הראשון למלבן עבה ולא גדול ובעזרת גלגלת פיצה נחתוך לריבועים
+כל ריבוע נגלגל לכדור
 נטבול כל כדור בחמאה ואז בתערובת של הסוכר והקינמון
 נסדר את הכדורים תבנית עגולה כאשר באמצע שמנו קערה קטנה (לא חייב אפשר גם לשים בקערה מחוץ לתבנית זה נטו ליופי)
 נתפיח את הכדורים בתבנית בחוץ 40-60 דקות
 ואז נאפה בתנור שחומם מראש על טורבו 170 מעלות ל35-45 מעלות
-כשהכדורים יוצאים מהתנור נערבב בתוך הקערית את האבקת סוכר והחלב 
+כשהכדורים יוצאים מהתנור נערבב בתוך הקערית את האבקת סוכר והחלב
 נטבול כל כדור ברוטב ובתאבון ❤️❤️</x:t>
         </x:is>
       </x:c>

</xml_diff>